<commit_message>
feat: Enhance Excel/CSV import functionality and UI
- Implemented a new import mode selection with radio buttons for "append" and "replace".
- Improved user feedback during import with detailed messages for skipped rows and invalid attachments.
- Added template validation to ensure uploaded files conform to the required structure.
- Refactored the import rendering logic to improve clarity and maintainability.
- Introduced a new single-select dropdown UI component for better user experience.
- Updated deduplication logic in the backend to consider distinct attachments.
- Enhanced test coverage for deduplication scenarios and whitespace handling.
</commit_message>
<xml_diff>
--- a/resource/template.xlsx
+++ b/resource/template.xlsx
@@ -27,30 +27,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
-    <t>序号</t>
+    <t>编号</t>
   </si>
   <si>
     <t>场景</t>
   </si>
   <si>
-    <t>学科</t>
-  </si>
-  <si>
     <t>难度</t>
   </si>
   <si>
-    <t>输入类型</t>
-  </si>
-  <si>
-    <t>是否本Agent强项</t>
-  </si>
-  <si>
     <t>Query内容</t>
-  </si>
-  <si>
-    <t>Skill</t>
   </si>
   <si>
     <t>附件</t>
@@ -59,16 +47,7 @@
     <t>备课</t>
   </si>
   <si>
-    <t>数学</t>
-  </si>
-  <si>
-    <t>进阶</t>
-  </si>
-  <si>
-    <t>带附件</t>
-  </si>
-  <si>
-    <t>否</t>
+    <t>易/中/难</t>
   </si>
   <si>
     <t>请帮我重构教学过程写到我原来的模板里，其他部分不要变。</t>
@@ -76,11 +55,14 @@
   <si>
     <t>小学数学教学设计.docx</t>
   </si>
+  <si>
+    <t>中</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
@@ -89,160 +71,160 @@
   </numFmts>
   <fonts count="21">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="PingFang SC Regular"/>
       <charset val="134"/>
-    </font>
-    <font>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
       <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
       <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -551,148 +533,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="false" applyFont="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -700,14 +682,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -953,8 +935,8 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+  <tableStyles count="2" defaultPivotStyle="PivotStylePreset2_Accent1" defaultTableStyle="TableStylePreset3_Accent1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -963,7 +945,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+    <tableStyle name="PivotStylePreset2_Accent1" pivot="0" count="10">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -985,7 +967,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1236,6 +1218,7 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1245,68 +1228,45 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="9.64285714285714" defaultRowHeight="16.8" outlineLevelRow="1"/>
   <cols>
-    <col min="7" max="7" width="34.2232142857143" customWidth="1"/>
-    <col min="8" max="8" width="22.4642857142857" customWidth="1"/>
-    <col min="9" max="9" width="27.6785714285714" customWidth="1"/>
+    <col customWidth="true" max="3" min="3" width="46.2767857142857"/>
+    <col customWidth="true" max="4" min="4" width="27.6785714285714"/>
+    <col customWidth="true" max="5" min="5" width="20.9821428571429"/>
+    <col customWidth="true" max="6" min="6" width="34.2232142857143"/>
+    <col customWidth="true" max="7" min="7" width="22.4642857142857"/>
+    <col customWidth="true" max="8" min="8" width="27.6785714285714"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="1"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" ht="118">
+      <c r="A2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2"/>
-    </row>
-    <row r="2" ht="34" spans="1:10">
-      <c r="A2" s="1">
-        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="2"/>
+      <c r="E2" s="1"/>
+      <c r="I2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>